<commit_message>
call a module's highest-kME proteins its top members instead of hubs
</commit_message>
<xml_diff>
--- a/02_HRvLR_groups/Figures/F2_Programmes/c_data/f2_programmes.xlsx
+++ b/02_HRvLR_groups/Figures/F2_Programmes/c_data/f2_programmes.xlsx
@@ -45,7 +45,7 @@
     <t>panel_a</t>
   </si>
   <si>
-    <t>a: module size, top set and its FDR, three hub proteins, STRING enrichment ratio.</t>
+    <t>a: module size, top set and its FDR, three top members, STRING enrichment ratio.</t>
   </si>
   <si>
     <t>panel_b</t>
@@ -135,7 +135,7 @@
     <t>FDR of the top set.</t>
   </si>
   <si>
-    <t>hubs</t>
+    <t>top_members</t>
   </si>
   <si>
     <t>Members with the highest kME.</t>
@@ -273,10 +273,10 @@
     <t>a</t>
   </si>
   <si>
-    <t>module size, top set and hubs</t>
-  </si>
-  <si>
-    <t>01_Trunk/07_Module_Characterisation/c_data/module_characterisation.xlsx</t>
+    <t>module size, top set and top members</t>
+  </si>
+  <si>
+    <t>01_Processing/07_Module_Characterisation/c_data/module_characterisation.xlsx</t>
   </si>
   <si>
     <t>labels</t>
@@ -321,7 +321,7 @@
     <t>eigengene per person</t>
   </si>
   <si>
-    <t>01_Trunk/06_Module_Building/c_data/modules.rds</t>
+    <t>01_Processing/06_Module_Building/c_data/modules.rds</t>
   </si>
   <si>
     <t>eigengenes</t>
@@ -615,7 +615,7 @@
     <t>module_labels</t>
   </si>
   <si>
-    <t>4b9f7cd5493b79c191734d7421f3b125</t>
+    <t>3a59bd479a4ab3c42392acd8f78f3eaf</t>
   </si>
   <si>
     <t>BiocGenerics</t>

</xml_diff>